<commit_message>
🔄 Index Monitor Update - 2026-10-02 07:55:34 UTC
Detected 6 going-forward index changes

Automated commit by GitHub Actions
</commit_message>
<xml_diff>
--- a/index_changes_evidence.xlsx
+++ b/index_changes_evidence.xlsx
@@ -438,7 +438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J51"/>
+  <dimension ref="A1:J54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -942,22 +942,34 @@
           <t>2026-06-11</t>
         </is>
       </c>
-      <c r="E10" s="2" t="inlineStr"/>
-      <c r="F10" s="2" t="inlineStr"/>
-      <c r="G10" s="2" t="inlineStr"/>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>Corteva</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>CTVA</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>Removed, no matching addition found</t>
+          <t>Different effective dates — paired for reference only</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>Merger/Acquisition: (NYSE: DHR ) is acquiring Masimo in a deal expected to be completed soon pending final conditions.</t>
+          <t>Spin-off: (NYSE: VYLR ) was added to the S&amp;P 500 on October 1 when S&amp;P 500 constituent Corteva Inc (NYSE: CTVA ) spun off Vylor in a transaction completed on that date. | Merger/Acquisition: (NYSE: DHR ) is acquiring Masimo in a deal expected to be completed soon pending final conditions.</t>
         </is>
       </c>
       <c r="J10" s="3" t="inlineStr">
         <is>
-          <t>https://www.prnewswire.com/news-releases/sirius-xm-holdings-set-to-join-sp-midcap-400-302794483.html</t>
+          <t>https://www.prnewswire.com/news-releases/vylor-added-to-the-sp-500-twilio-set-to-join-sp-500-others-to-join-sp-midcap-400-and-sp-smallcap-600-302896675.html</t>
         </is>
       </c>
     </row>
@@ -1194,22 +1206,34 @@
           <t>2026-08-18</t>
         </is>
       </c>
-      <c r="E16" s="2" t="inlineStr"/>
-      <c r="F16" s="2" t="inlineStr"/>
-      <c r="G16" s="2" t="inlineStr"/>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>Vylor</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>VYLR</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>Removed, no matching addition found</t>
+          <t>Different effective dates — paired for reference only</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>Merger/Acquisition: S&amp;P 500 constituent Equity Residential (NYSE: EQR ) is acquiring AvalonBay Communities in a deal expected to be completed soon, pending final conditions.</t>
+          <t>Spin-off: (NYSE: VYLR ) was added to the S&amp;P 500 on October 1 when S&amp;P 500 constituent Corteva Inc (NYSE: CTVA ) spun off Vylor in a transaction completed on that date. | Merger/Acquisition: S&amp;P 500 constituent Equity Residential (NYSE: EQR ) is acquiring AvalonBay Communities in a deal expected to be completed soon, pending final conditions.</t>
         </is>
       </c>
       <c r="J16" s="3" t="inlineStr">
         <is>
-          <t>https://www.prnewswire.com/news-releases/reddit-set-to-join-sp-500-and-sun-communities-to-join-sp-midcap-400-302851432.html</t>
+          <t>https://www.prnewswire.com/news-releases/vylor-added-to-the-sp-500-twilio-set-to-join-sp-500-others-to-join-sp-midcap-400-and-sp-smallcap-600-302896675.html</t>
         </is>
       </c>
     </row>
@@ -1256,104 +1280,80 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>S&amp;P 600</t>
+          <t>S&amp;P 500</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Brandywine Realty Trust</t>
+          <t>Corteva</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>BDN</t>
+          <t>CTVA</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
-        </is>
-      </c>
-      <c r="E18" s="2" t="inlineStr">
-        <is>
-          <t>Versant Media Group</t>
-        </is>
-      </c>
-      <c r="F18" s="2" t="inlineStr">
-        <is>
-          <t>VSNT</t>
-        </is>
-      </c>
-      <c r="G18" s="2" t="inlineStr">
-        <is>
-          <t>2026-01-07</t>
-        </is>
-      </c>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr"/>
+      <c r="F18" s="2" t="inlineStr"/>
+      <c r="G18" s="2" t="inlineStr"/>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>Same effective date</t>
+          <t>Removed, no matching addition found</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>Spin-off: VSNT was spun off fromComcastand replaced BDN which was no longer representative of the small-cap market space.[38]</t>
+          <t>Spin-off: (NYSE: VYLR ) was added to the S&amp;P 500 on October 1 when S&amp;P 500 constituent Corteva Inc (NYSE: CTVA ) spun off Vylor in a transaction completed on that date.</t>
         </is>
       </c>
       <c r="J18" s="3" t="inlineStr">
         <is>
-          <t>https://en.wikipedia.org/wiki/List_of_S%26P_600_companies</t>
+          <t>https://www.prnewswire.com/news-releases/vylor-added-to-the-sp-500-twilio-set-to-join-sp-500-others-to-join-sp-midcap-400-and-sp-smallcap-600-302896675.html</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>S&amp;P 600</t>
+          <t>S&amp;P 500</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Guess, Inc.</t>
+          <t>Warner Bros. Discovery</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>GES</t>
+          <t>WBD</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>2026-01-26</t>
-        </is>
-      </c>
-      <c r="E19" s="2" t="inlineStr">
-        <is>
-          <t>Winmark</t>
-        </is>
-      </c>
-      <c r="F19" s="2" t="inlineStr">
-        <is>
-          <t>WINA</t>
-        </is>
-      </c>
-      <c r="G19" s="2" t="inlineStr">
-        <is>
-          <t>2026-01-26</t>
-        </is>
-      </c>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr"/>
+      <c r="F19" s="2" t="inlineStr"/>
+      <c r="G19" s="2" t="inlineStr"/>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>Same effective date</t>
+          <t>Removed, no matching addition found</t>
         </is>
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>Merger/Acquisition: WINA replaced GES after it was acquired byAuthentic Brands Groupand the Rolling Stockholders.[37]</t>
+          <t>Merger/Acquisition: (NASD: PSKY) is acquiring Warner Bros.</t>
         </is>
       </c>
       <c r="J19" s="3" t="inlineStr">
         <is>
-          <t>https://en.wikipedia.org/wiki/List_of_S%26P_600_companies</t>
+          <t>https://www.prnewswire.com/news-releases/vylor-added-to-the-sp-500-twilio-set-to-join-sp-500-others-to-join-sp-midcap-400-and-sp-smallcap-600-302896675.html</t>
         </is>
       </c>
     </row>
@@ -1365,32 +1365,32 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>TTM Technologies</t>
+          <t>Brandywine Realty Trust</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>TTMI</t>
+          <t>BDN</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>2026-01-30</t>
+          <t>2026-01-07</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>Amneal Pharmaceuticals</t>
+          <t>Versant Media Group</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>AMRX</t>
+          <t>VSNT</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>2026-01-30</t>
+          <t>2026-01-07</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
@@ -1400,7 +1400,7 @@
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>Merger/Acquisition: AMRX replaced TTMI, which replaced Civitas Resources in theS&amp;P 400after it was acquired bySM Energy.[36]</t>
+          <t>Spin-off: VSNT was spun off fromComcastand replaced BDN which was no longer representative of the small-cap market space.[38]</t>
         </is>
       </c>
       <c r="J20" s="3" t="inlineStr">
@@ -1417,32 +1417,32 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Advanced Energy</t>
+          <t>Guess, Inc.</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>AEIS</t>
+          <t>GES</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>2026-02-02</t>
+          <t>2026-01-26</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>Apellis Pharmaceuticals</t>
+          <t>Winmark</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>APLS</t>
+          <t>WINA</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>2026-02-02</t>
+          <t>2026-01-26</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
@@ -1452,7 +1452,7 @@
       </c>
       <c r="I21" s="2" t="inlineStr">
         <is>
-          <t>Merger/Acquisition: APLS replaced AEIS, which replacedComericain the S&amp;P 400 after it was acquired byFifth Third Bank.[36]</t>
+          <t>Merger/Acquisition: WINA replaced GES after it was acquired byAuthentic Brands Groupand the Rolling Stockholders.[37]</t>
         </is>
       </c>
       <c r="J21" s="3" t="inlineStr">
@@ -1469,32 +1469,32 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Dynavax Technologies</t>
+          <t>TTM Technologies</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>DVAX</t>
+          <t>TTMI</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>2026-02-10</t>
+          <t>2026-01-30</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>OneSpaWorld Holdings</t>
+          <t>Amneal Pharmaceuticals</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>OSW</t>
+          <t>AMRX</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>2026-02-10</t>
+          <t>2026-01-30</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
@@ -1504,7 +1504,7 @@
       </c>
       <c r="I22" s="2" t="inlineStr">
         <is>
-          <t>Merger/Acquisition: OSW replaced DVAX after it was acquired bySanofi.[35]</t>
+          <t>Merger/Acquisition: AMRX replaced TTMI, which replaced Civitas Resources in theS&amp;P 400after it was acquired bySM Energy.[36]</t>
         </is>
       </c>
       <c r="J22" s="3" t="inlineStr">
@@ -1521,32 +1521,32 @@
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>TreeHouse Foods</t>
+          <t>Advanced Energy</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>THS</t>
+          <t>AEIS</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>2026-02-11</t>
+          <t>2026-02-02</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>Merchants Bancorp</t>
+          <t>Apellis Pharmaceuticals</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>MBIN</t>
+          <t>APLS</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>2026-02-11</t>
+          <t>2026-02-02</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
@@ -1556,7 +1556,7 @@
       </c>
       <c r="I23" s="2" t="inlineStr">
         <is>
-          <t>Merger/Acquisition: MBIN replaced THS after it was acquired by Investindustrial S.A.[34]</t>
+          <t>Merger/Acquisition: APLS replaced AEIS, which replacedComericain the S&amp;P 400 after it was acquired byFifth Third Bank.[36]</t>
         </is>
       </c>
       <c r="J23" s="3" t="inlineStr">
@@ -1573,32 +1573,32 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>Hillenbrand</t>
+          <t>Dynavax Technologies</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>HI</t>
+          <t>DVAX</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>2026-02-12</t>
+          <t>2026-02-10</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>RingCentral</t>
+          <t>OneSpaWorld Holdings</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>RNG</t>
+          <t>OSW</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>2026-02-12</t>
+          <t>2026-02-10</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr">
@@ -1608,7 +1608,7 @@
       </c>
       <c r="I24" s="2" t="inlineStr">
         <is>
-          <t>Merger/Acquisition: RNG replaced HI after it was acquired byLone Star Funds.[33]</t>
+          <t>Merger/Acquisition: OSW replaced DVAX after it was acquired bySanofi.[35]</t>
         </is>
       </c>
       <c r="J24" s="3" t="inlineStr">
@@ -1625,32 +1625,32 @@
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>Alexander &amp; Baldwin</t>
+          <t>TreeHouse Foods</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>ALEX</t>
+          <t>THS</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>2026-03-13</t>
+          <t>2026-02-11</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>Napco Security Technologies</t>
+          <t>Merchants Bancorp</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>NSSC</t>
+          <t>MBIN</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>2026-03-13</t>
+          <t>2026-02-11</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
@@ -1660,7 +1660,7 @@
       </c>
       <c r="I25" s="2" t="inlineStr">
         <is>
-          <t>Merger/Acquisition: NSSC replaced ALEX after it was acquired by an investor group comprising MW Group and funds affiliated with DivcoWest andBlackstone Real Estate.[32]</t>
+          <t>Merger/Acquisition: MBIN replaced THS after it was acquired by Investindustrial S.A.[34]</t>
         </is>
       </c>
       <c r="J25" s="3" t="inlineStr">
@@ -1677,32 +1677,32 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>Tegna Inc.</t>
+          <t>Hillenbrand</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>TGNA</t>
+          <t>HI</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-02-12</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>Vita Coco</t>
+          <t>RingCentral</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>COCO</t>
+          <t>RNG</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-02-12</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr">
@@ -1712,7 +1712,7 @@
       </c>
       <c r="I26" s="2" t="inlineStr">
         <is>
-          <t>Merger/Acquisition: COCO replaced TGNA after it was acquired byNexstar Media Group.[31]</t>
+          <t>Merger/Acquisition: RNG replaced HI after it was acquired byLone Star Funds.[33]</t>
         </is>
       </c>
       <c r="J26" s="3" t="inlineStr">
@@ -1729,32 +1729,32 @@
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>Titan International, Inc.</t>
+          <t>Alexander &amp; Baldwin</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>TWI</t>
+          <t>ALEX</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-03-13</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>Versigent</t>
+          <t>Napco Security Technologies</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>VGNT</t>
+          <t>NSSC</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-03-13</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr">
@@ -1764,7 +1764,7 @@
       </c>
       <c r="I27" s="2" t="inlineStr">
         <is>
-          <t>Spin-off: VGNT was spun off fromAptivand replaced TWI which was no longer representative of the small-cap market space.[30]</t>
+          <t>Merger/Acquisition: NSSC replaced ALEX after it was acquired by an investor group comprising MW Group and funds affiliated with DivcoWest andBlackstone Real Estate.[32]</t>
         </is>
       </c>
       <c r="J27" s="3" t="inlineStr">
@@ -1781,32 +1781,32 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>Air Lease Corporation</t>
+          <t>Tegna Inc.</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>AL</t>
+          <t>TGNA</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>Atmus Filtration Technologies</t>
+          <t>Vita Coco</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>ATMU</t>
+          <t>COCO</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr">
@@ -1816,7 +1816,7 @@
       </c>
       <c r="I28" s="2" t="inlineStr">
         <is>
-          <t>Merger/Acquisition: ATMU replaced AL after it was acquired bySumitomo Corporation.[29]</t>
+          <t>Merger/Acquisition: COCO replaced TGNA after it was acquired byNexstar Media Group.[31]</t>
         </is>
       </c>
       <c r="J28" s="3" t="inlineStr">
@@ -1833,32 +1833,32 @@
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>Sealed Air</t>
+          <t>Titan International, Inc.</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>SEE</t>
+          <t>TWI</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-02</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>Diebold Nixdorf</t>
+          <t>Versigent</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>DBD</t>
+          <t>VGNT</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-02</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -1868,7 +1868,7 @@
       </c>
       <c r="I29" s="2" t="inlineStr">
         <is>
-          <t>Merger/Acquisition: DBD replaced SEE after it was acquired byClayton, Dubilier &amp; Rice.[27]</t>
+          <t>Spin-off: VGNT was spun off fromAptivand replaced TWI which was no longer representative of the small-cap market space.[30]</t>
         </is>
       </c>
       <c r="J29" s="3" t="inlineStr">
@@ -1885,32 +1885,32 @@
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>Golden Entertainment</t>
+          <t>Air Lease Corporation</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>GDEN</t>
+          <t>AL</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>Lifestance Health</t>
+          <t>Atmus Filtration Technologies</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>LFST</t>
+          <t>ATMU</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -1920,7 +1920,7 @@
       </c>
       <c r="I30" s="2" t="inlineStr">
         <is>
-          <t>Merger/Acquisition: LFST replaced GDEN after it was acquired byVici PropertiesandBlake L. Sartini.[25]</t>
+          <t>Merger/Acquisition: ATMU replaced AL after it was acquired bySumitomo Corporation.[29]</t>
         </is>
       </c>
       <c r="J30" s="3" t="inlineStr">
@@ -1937,32 +1937,32 @@
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>Apellis Pharmaceuticals</t>
+          <t>Sealed Air</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>APLS</t>
+          <t>SEE</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>Alignment Healthcare</t>
+          <t>Diebold Nixdorf</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>ALHC</t>
+          <t>DBD</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr">
@@ -1972,7 +1972,7 @@
       </c>
       <c r="I31" s="2" t="inlineStr">
         <is>
-          <t>Merger/Acquisition: ALHC replaced SNCY after it was acquired byAllegiant Travel Company.[22] | Merger/Acquisition: RELY replaced APLS after it was acquired byBiogen.[23]</t>
+          <t>Merger/Acquisition: DBD replaced SEE after it was acquired byClayton, Dubilier &amp; Rice.[27]</t>
         </is>
       </c>
       <c r="J31" s="3" t="inlineStr">
@@ -1989,32 +1989,32 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>Sun Country Airlines</t>
+          <t>Golden Entertainment</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>SNCY</t>
+          <t>GDEN</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>Bright Horizons</t>
+          <t>Lifestance Health</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>BFAM</t>
+          <t>LFST</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr">
@@ -2024,7 +2024,7 @@
       </c>
       <c r="I32" s="2" t="inlineStr">
         <is>
-          <t>Merger/Acquisition: BFAM replaced TPH after it was acquired bySumitomo Forestry.[23] | Merger/Acquisition: ALHC replaced SNCY after it was acquired byAllegiant Travel Company.[22]</t>
+          <t>Merger/Acquisition: LFST replaced GDEN after it was acquired byVici PropertiesandBlake L. Sartini.[25]</t>
         </is>
       </c>
       <c r="J32" s="3" t="inlineStr">
@@ -2041,12 +2041,12 @@
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>Tri Pointe Homes</t>
+          <t>Apellis Pharmaceuticals</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>TPH</t>
+          <t>APLS</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
@@ -2056,12 +2056,12 @@
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>Remitly</t>
+          <t>Alignment Healthcare</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>RELY</t>
+          <t>ALHC</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
@@ -2076,7 +2076,7 @@
       </c>
       <c r="I33" s="2" t="inlineStr">
         <is>
-          <t>Merger/Acquisition: RELY replaced APLS after it was acquired byBiogen.[23] | Merger/Acquisition: BFAM replaced TPH after it was acquired bySumitomo Forestry.[23]</t>
+          <t>Merger/Acquisition: ALHC replaced SNCY after it was acquired byAllegiant Travel Company.[22] | Merger/Acquisition: RELY replaced APLS after it was acquired byBiogen.[23]</t>
         </is>
       </c>
       <c r="J33" s="3" t="inlineStr">
@@ -2093,32 +2093,32 @@
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>CSG Systems</t>
+          <t>Sun Country Airlines</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>CSGS</t>
+          <t>SNCY</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>Flowers Foods</t>
+          <t>Bright Horizons</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>FLO</t>
+          <t>BFAM</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr">
@@ -2128,7 +2128,7 @@
       </c>
       <c r="I34" s="2" t="inlineStr">
         <is>
-          <t>Merger/Acquisition: FLO replaced CSGS after it was acquired byNEC.[21]</t>
+          <t>Merger/Acquisition: BFAM replaced TPH after it was acquired bySumitomo Forestry.[23] | Merger/Acquisition: ALHC replaced SNCY after it was acquired byAllegiant Travel Company.[22]</t>
         </is>
       </c>
       <c r="J34" s="3" t="inlineStr">
@@ -2145,32 +2145,32 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>Enviri</t>
+          <t>Tri Pointe Homes</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>NVRI</t>
+          <t>TPH</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>Peloton Interactive</t>
+          <t>Remitly</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>PTON</t>
+          <t>RELY</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="H35" s="2" t="inlineStr">
@@ -2180,7 +2180,7 @@
       </c>
       <c r="I35" s="2" t="inlineStr">
         <is>
-          <t>Spin-off: PTON replaced NVRI after it spun off assets into a new publicly traded company. The new publicly traded company was not representative of the small-cap market space.[20]</t>
+          <t>Merger/Acquisition: RELY replaced APLS after it was acquired byBiogen.[23] | Merger/Acquisition: BFAM replaced TPH after it was acquired bySumitomo Forestry.[23]</t>
         </is>
       </c>
       <c r="J35" s="3" t="inlineStr">
@@ -2197,32 +2197,32 @@
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>Mister Car Wash</t>
+          <t>CSG Systems</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>MCW</t>
+          <t>CSGS</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>F&amp;G</t>
+          <t>Flowers Foods</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>FG</t>
+          <t>FLO</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr">
@@ -2232,7 +2232,7 @@
       </c>
       <c r="I36" s="2" t="inlineStr">
         <is>
-          <t>Merger/Acquisition: FG replaced MCW after it was acquired byLeonard Green &amp; Partners.[21]</t>
+          <t>Merger/Acquisition: FLO replaced CSGS after it was acquired byNEC.[21]</t>
         </is>
       </c>
       <c r="J36" s="3" t="inlineStr">
@@ -2249,32 +2249,32 @@
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>Veris Residential</t>
+          <t>Enviri</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>VRE</t>
+          <t>NVRI</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>Universal Technical Institute</t>
+          <t>Peloton Interactive</t>
         </is>
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>UTI</t>
+          <t>PTON</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="H37" s="2" t="inlineStr">
@@ -2284,7 +2284,7 @@
       </c>
       <c r="I37" s="2" t="inlineStr">
         <is>
-          <t>Merger/Acquisition: UTI replaced VRE after it was acquired by Affinius Capital and Vista Hill Partners.[20]</t>
+          <t>Spin-off: PTON replaced NVRI after it spun off assets into a new publicly traded company. The new publicly traded company was not representative of the small-cap market space.[20]</t>
         </is>
       </c>
       <c r="J37" s="3" t="inlineStr">
@@ -2301,32 +2301,32 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>American Woodmark</t>
+          <t>Mister Car Wash</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>AMWD</t>
+          <t>MCW</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>Dave</t>
+          <t>F&amp;G</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>DAVE</t>
+          <t>FG</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="H38" s="2" t="inlineStr">
@@ -2336,7 +2336,7 @@
       </c>
       <c r="I38" s="2" t="inlineStr">
         <is>
-          <t>Merger/Acquisition: DAVE replaced AMWD after it was acquired by MasterBrand Inc.[19]</t>
+          <t>Merger/Acquisition: FG replaced MCW after it was acquired byLeonard Green &amp; Partners.[21]</t>
         </is>
       </c>
       <c r="J38" s="3" t="inlineStr">
@@ -2353,32 +2353,32 @@
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>Shutterstock</t>
+          <t>Veris Residential</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>SSTK</t>
+          <t>VRE</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>EPAM Systems</t>
+          <t>Universal Technical Institute</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>EPAM</t>
+          <t>UTI</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="H39" s="2" t="inlineStr">
@@ -2388,7 +2388,7 @@
       </c>
       <c r="I39" s="2" t="inlineStr">
         <is>
-          <t>Merger/Acquisition: EPAM was moved from theS&amp;P 500as it was more representative of the small cap market space. SSTK was removed from theS&amp;P 600as it was merged withGetty Images.[19]</t>
+          <t>Merger/Acquisition: UTI replaced VRE after it was acquired by Affinius Capital and Vista Hill Partners.[20]</t>
         </is>
       </c>
       <c r="J39" s="3" t="inlineStr">
@@ -2405,32 +2405,32 @@
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>Core Laboratories</t>
+          <t>American Woodmark</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>CLB</t>
+          <t>AMWD</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>Mobility Global</t>
+          <t>Dave</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>MBGL</t>
+          <t>DAVE</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr">
@@ -2440,7 +2440,7 @@
       </c>
       <c r="I40" s="2" t="inlineStr">
         <is>
-          <t>Spin-off: MBGL was spun off fromS&amp;P Globaland replaced CLB which was no longer representative of the small-cap market space.[13]</t>
+          <t>Merger/Acquisition: DAVE replaced AMWD after it was acquired by MasterBrand Inc.[19]</t>
         </is>
       </c>
       <c r="J40" s="3" t="inlineStr">
@@ -2457,32 +2457,32 @@
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>Whitestone REIT</t>
+          <t>Shutterstock</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>WSR</t>
+          <t>SSTK</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>Centrus Energy</t>
+          <t>EPAM Systems</t>
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>LEU</t>
+          <t>EPAM</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="H41" s="2" t="inlineStr">
@@ -2492,7 +2492,7 @@
       </c>
       <c r="I41" s="2" t="inlineStr">
         <is>
-          <t>Merger/Acquisition: LEU replaced WSR after it was acquired byAres Management.[11]</t>
+          <t>Merger/Acquisition: EPAM was moved from theS&amp;P 500as it was more representative of the small cap market space. SSTK was removed from theS&amp;P 600as it was merged withGetty Images.[19]</t>
         </is>
       </c>
       <c r="J41" s="3" t="inlineStr">
@@ -2509,32 +2509,32 @@
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>Hertz Global Holdings</t>
+          <t>Core Laboratories</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>HTZ</t>
+          <t>CLB</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>ADI Global Distribution</t>
+          <t>Mobility Global</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>ADIG</t>
+          <t>MBGL</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr">
@@ -2544,12 +2544,12 @@
       </c>
       <c r="I42" s="2" t="inlineStr">
         <is>
-          <t>Merger/Acquisition: News in Focus Browse News Releases All News Releases All Public Company English-only News Releases Overview Multimedia Gallery All Multimedia All Photos All Videos Multimedia Gallery Overview Trending Topics All Trending Topics Business &amp; Money Auto &amp; Transportation All Automo... | Spin-off: ADIG was spun off fromResideoand replaced HTZ which was no longer representative of the small-cap market space.[5]</t>
+          <t>Spin-off: MBGL was spun off fromS&amp;P Globaland replaced CLB which was no longer representative of the small-cap market space.[13]</t>
         </is>
       </c>
       <c r="J42" s="3" t="inlineStr">
         <is>
-          <t>https://www.prnewswire.com/news-releases/ferguson-enterprises-set-to-join-sp-500-and-adi-global-distribution-to-join-sp-smallcap-600-302840407.html</t>
+          <t>https://en.wikipedia.org/wiki/List_of_S%26P_600_companies</t>
         </is>
       </c>
     </row>
@@ -2561,47 +2561,47 @@
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>Kennedy-Wilson Holdings</t>
+          <t>Whitestone REIT</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>KW</t>
+          <t>WSR</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>National Health Investors</t>
+          <t>Centrus Energy</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>NHI</t>
+          <t>LEU</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="H43" s="2" t="inlineStr">
         <is>
-          <t>Different effective dates — paired for reference only</t>
+          <t>Same effective date</t>
         </is>
       </c>
       <c r="I43" s="2" t="inlineStr">
         <is>
-          <t>Merger/Acquisition: News in Focus Browse News Releases All News Releases All Public Company English-only News Releases Overview Multimedia Gallery All Multimedia All Photos All Videos Multimedia Gallery Overview Trending Topics All Trending Topics Business &amp; Money Auto &amp; Transportation All Automo... | Merger/Acquisition: A consortium led by KW's CEO with Fairfax Financial Holdings Limited (TSE: FFH) is acquiring Kennedy-Wilson Holdings in a deal expected to close soon, pending final closing conditions.</t>
+          <t>Merger/Acquisition: LEU replaced WSR after it was acquired byAres Management.[11]</t>
         </is>
       </c>
       <c r="J43" s="3" t="inlineStr">
         <is>
-          <t>https://www.prnewswire.com/news-releases/honeywell-aerospace-set-to-join-sp-500--sp-100-others-to-join-sp-midcap-400-and-sp-smallcap-600-302808386.html</t>
+          <t>https://en.wikipedia.org/wiki/List_of_S%26P_600_companies</t>
         </is>
       </c>
     </row>
@@ -2613,47 +2613,47 @@
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>ProAssurance</t>
+          <t>Hertz Global Holdings</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>PRA</t>
+          <t>HTZ</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>Construction Partners</t>
+          <t>ADI Global Distribution</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>ROAD</t>
+          <t>ADIG</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="H44" s="2" t="inlineStr">
         <is>
-          <t>Different effective dates — paired for reference only</t>
+          <t>Same effective date</t>
         </is>
       </c>
       <c r="I44" s="2" t="inlineStr">
         <is>
-          <t>Merger/Acquisition: News in Focus Browse News Releases All News Releases All Public Company English-only News Releases Overview Multimedia Gallery All Multimedia All Photos All Videos Multimedia Gallery Overview Trending Topics All Trending Topics Business &amp; Money Auto &amp; Transportation All Automo... | Merger/Acquisition: The Doctors Company is acquiring ProAssurance in a cash deal expected to close soon, pending final closing conditions.</t>
+          <t>Merger/Acquisition: News in Focus Browse News Releases All News Releases All Public Company English-only News Releases Overview Multimedia Gallery All Multimedia All Photos All Videos Multimedia Gallery Overview Trending Topics All Trending Topics Business &amp; Money Auto &amp; Transportation All Automo... | Spin-off: ADIG was spun off fromResideoand replaced HTZ which was no longer representative of the small-cap market space.[5]</t>
         </is>
       </c>
       <c r="J44" s="3" t="inlineStr">
         <is>
-          <t>https://www.prnewswire.com/news-releases/molina-healthcare-set-to-join-sp-midcap-400-and-construction-partners-to-join-sp-smallcap-600-302828046.html</t>
+          <t>https://www.prnewswire.com/news-releases/ferguson-enterprises-set-to-join-sp-500-and-adi-global-distribution-to-join-sp-smallcap-600-302840407.html</t>
         </is>
       </c>
     </row>
@@ -2665,32 +2665,32 @@
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>Select Medical Holdings</t>
+          <t>Kennedy-Wilson Holdings</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>SEM</t>
+          <t>KW</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>The Trade Desk</t>
+          <t>National Health Investors</t>
         </is>
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>TTD</t>
+          <t>NHI</t>
         </is>
       </c>
       <c r="G45" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="H45" s="2" t="inlineStr">
@@ -2700,12 +2700,12 @@
       </c>
       <c r="I45" s="2" t="inlineStr">
         <is>
-          <t>Merger/Acquisition: News in Focus Browse News Releases All News Releases All Public Company English-only News Releases Overview Multimedia Gallery All Multimedia All Photos All Videos Multimedia Gallery Overview Trending Topics All Trending Topics Business &amp; Money Auto &amp; Transportation All Automo... | Merger/Acquisition: Select Medical Holdings is being acquired in a deal expected to be completed soon, pending final closing conditions.</t>
+          <t>Merger/Acquisition: News in Focus Browse News Releases All News Releases All Public Company English-only News Releases Overview Multimedia Gallery All Multimedia All Photos All Videos Multimedia Gallery Overview Trending Topics All Trending Topics Business &amp; Money Auto &amp; Transportation All Automo... | Merger/Acquisition: A consortium led by KW's CEO with Fairfax Financial Holdings Limited (TSE: FFH) is acquiring Kennedy-Wilson Holdings in a deal expected to close soon, pending final closing conditions.</t>
         </is>
       </c>
       <c r="J45" s="3" t="inlineStr">
         <is>
-          <t>https://www.prnewswire.com/news-releases/bloom-energy-illumina-and-everpure-set-to-join-sp-500-others-to-join-sp-100-sp-midcap-400-and-sp-smallcap-600-302870517.html</t>
+          <t>https://www.prnewswire.com/news-releases/honeywell-aerospace-set-to-join-sp-500--sp-100-others-to-join-sp-midcap-400-and-sp-smallcap-600-302808386.html</t>
         </is>
       </c>
     </row>
@@ -2717,35 +2717,47 @@
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>Stellar Bancorp</t>
+          <t>ProAssurance</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>STEL</t>
+          <t>PRA</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
-        </is>
-      </c>
-      <c r="E46" s="2" t="inlineStr"/>
-      <c r="F46" s="2" t="inlineStr"/>
-      <c r="G46" s="2" t="inlineStr"/>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="E46" s="2" t="inlineStr">
+        <is>
+          <t>Construction Partners</t>
+        </is>
+      </c>
+      <c r="F46" s="2" t="inlineStr">
+        <is>
+          <t>ROAD</t>
+        </is>
+      </c>
+      <c r="G46" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
       <c r="H46" s="2" t="inlineStr">
         <is>
-          <t>Removed, no matching addition found</t>
+          <t>Different effective dates — paired for reference only</t>
         </is>
       </c>
       <c r="I46" s="2" t="inlineStr">
         <is>
-          <t>Merger/Acquisition: (NYSE: PB ) is acquiring Stellar Bancorp in a deal expected to close July 1.</t>
+          <t>Merger/Acquisition: News in Focus Browse News Releases All News Releases All Public Company English-only News Releases Overview Multimedia Gallery All Multimedia All Photos All Videos Multimedia Gallery Overview Trending Topics All Trending Topics Business &amp; Money Auto &amp; Transportation All Automo... | Merger/Acquisition: The Doctors Company is acquiring ProAssurance in a cash deal expected to close soon, pending final closing conditions.</t>
         </is>
       </c>
       <c r="J46" s="3" t="inlineStr">
         <is>
-          <t>https://www.prnewswire.com/news-releases/allison-transmission-holdings-set-to-join-sp-midcap-400-and-goodyear-tire--rubber-to-join-sp-smallcap-600-302815143.html</t>
+          <t>https://www.prnewswire.com/news-releases/molina-healthcare-set-to-join-sp-midcap-400-and-construction-partners-to-join-sp-smallcap-600-302828046.html</t>
         </is>
       </c>
     </row>
@@ -2757,35 +2769,47 @@
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>Whitestone REIT</t>
+          <t>Select Medical Holdings</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>WSR</t>
+          <t>SEM</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
-        </is>
-      </c>
-      <c r="E47" s="2" t="inlineStr"/>
-      <c r="F47" s="2" t="inlineStr"/>
-      <c r="G47" s="2" t="inlineStr"/>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="E47" s="2" t="inlineStr">
+        <is>
+          <t>The Trade Desk</t>
+        </is>
+      </c>
+      <c r="F47" s="2" t="inlineStr">
+        <is>
+          <t>TTD</t>
+        </is>
+      </c>
+      <c r="G47" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
       <c r="H47" s="2" t="inlineStr">
         <is>
-          <t>Removed, no matching addition found</t>
+          <t>Different effective dates — paired for reference only</t>
         </is>
       </c>
       <c r="I47" s="2" t="inlineStr">
         <is>
-          <t>Merger/Acquisition: (NYSE: ARES ) is acquiring Whitestone REIT in a deal expected to close on or about that date, pending final closing conditions.</t>
+          <t>Merger/Acquisition: News in Focus Browse News Releases All News Releases All Public Company English-only News Releases Overview Multimedia Gallery All Multimedia All Photos All Videos Multimedia Gallery Overview Trending Topics All Trending Topics Business &amp; Money Auto &amp; Transportation All Automo... | Merger/Acquisition: Select Medical Holdings is being acquired in a deal expected to be completed soon, pending final closing conditions.</t>
         </is>
       </c>
       <c r="J47" s="3" t="inlineStr">
         <is>
-          <t>https://www.prnewswire.com/news-releases/midera-food-processing-and-centrus-energy-set-to-join-sp-smallcap-600-302817273.html</t>
+          <t>https://www.prnewswire.com/news-releases/bloom-energy-illumina-and-everpure-set-to-join-sp-500-others-to-join-sp-100-sp-midcap-400-and-sp-smallcap-600-302870517.html</t>
         </is>
       </c>
     </row>
@@ -2797,17 +2821,17 @@
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>Catalyst Pharmaceuticals</t>
+          <t>Stellar Bancorp</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>CPRX</t>
+          <t>STEL</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr"/>
@@ -2820,12 +2844,12 @@
       </c>
       <c r="I48" s="2" t="inlineStr">
         <is>
-          <t>Merger/Acquisition: is acquiring Catalyst Pharmaceuticals in a deal expected to close soon, pending final closing conditions.</t>
+          <t>Merger/Acquisition: (NYSE: PB ) is acquiring Stellar Bancorp in a deal expected to close July 1.</t>
         </is>
       </c>
       <c r="J48" s="3" t="inlineStr">
         <is>
-          <t>https://www.prnewswire.com/news-releases/solaris-energy-infrastructure-set-to-join-sp-smallcap-600-302822362.html</t>
+          <t>https://www.prnewswire.com/news-releases/allison-transmission-holdings-set-to-join-sp-midcap-400-and-goodyear-tire--rubber-to-join-sp-smallcap-600-302815143.html</t>
         </is>
       </c>
     </row>
@@ -2837,17 +2861,17 @@
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>Avanos Medical</t>
+          <t>Whitestone REIT</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>AVNS</t>
+          <t>WSR</t>
         </is>
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="E49" s="2" t="inlineStr"/>
@@ -2860,12 +2884,12 @@
       </c>
       <c r="I49" s="2" t="inlineStr">
         <is>
-          <t>Merger/Acquisition: American Industrial Partners is acquiring Avanos Medical in a deal expected to close soon, pending final closing conditions.</t>
+          <t>Merger/Acquisition: (NYSE: ARES ) is acquiring Whitestone REIT in a deal expected to close on or about that date, pending final closing conditions.</t>
         </is>
       </c>
       <c r="J49" s="3" t="inlineStr">
         <is>
-          <t>https://www.prnewswire.com/news-releases/krystal-biotech-set-to-join-sp-midcap-400-tutor-perini-and-v2x-to-join-sp-smallcap-600-302830022.html</t>
+          <t>https://www.prnewswire.com/news-releases/midera-food-processing-and-centrus-energy-set-to-join-sp-smallcap-600-302817273.html</t>
         </is>
       </c>
     </row>
@@ -2877,17 +2901,17 @@
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>Two Harbors Investment</t>
+          <t>Catalyst Pharmaceuticals</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>TWO</t>
+          <t>CPRX</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="E50" s="2" t="inlineStr"/>
@@ -2900,12 +2924,12 @@
       </c>
       <c r="I50" s="2" t="inlineStr">
         <is>
-          <t>Merger/Acquisition: News in Focus Browse News Releases All News Releases All Public Company English-only News Releases Overview Multimedia Gallery All Multimedia All Photos All Videos Multimedia Gallery Overview Trending Topics All Trending Topics Business &amp; Money Auto &amp; Transportation All Automo...</t>
+          <t>Merger/Acquisition: is acquiring Catalyst Pharmaceuticals in a deal expected to close soon, pending final closing conditions.</t>
         </is>
       </c>
       <c r="J50" s="3" t="inlineStr">
         <is>
-          <t>https://www.prnewswire.com/news-releases/five9-set-to-join-sp-smallcap-600-302838329.html</t>
+          <t>https://www.prnewswire.com/news-releases/solaris-energy-infrastructure-set-to-join-sp-smallcap-600-302822362.html</t>
         </is>
       </c>
     </row>
@@ -2917,17 +2941,17 @@
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>Leggett &amp; Platt</t>
+          <t>Avanos Medical</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>LEG</t>
+          <t>AVNS</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="E51" s="2" t="inlineStr"/>
@@ -2940,12 +2964,132 @@
       </c>
       <c r="I51" s="2" t="inlineStr">
         <is>
+          <t>Merger/Acquisition: American Industrial Partners is acquiring Avanos Medical in a deal expected to close soon, pending final closing conditions.</t>
+        </is>
+      </c>
+      <c r="J51" s="3" t="inlineStr">
+        <is>
+          <t>https://www.prnewswire.com/news-releases/krystal-biotech-set-to-join-sp-midcap-400-tutor-perini-and-v2x-to-join-sp-smallcap-600-302830022.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>S&amp;P 600</t>
+        </is>
+      </c>
+      <c r="B52" s="2" t="inlineStr">
+        <is>
+          <t>Two Harbors Investment</t>
+        </is>
+      </c>
+      <c r="C52" s="2" t="inlineStr">
+        <is>
+          <t>TWO</t>
+        </is>
+      </c>
+      <c r="D52" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="E52" s="2" t="inlineStr"/>
+      <c r="F52" s="2" t="inlineStr"/>
+      <c r="G52" s="2" t="inlineStr"/>
+      <c r="H52" s="2" t="inlineStr">
+        <is>
+          <t>Removed, no matching addition found</t>
+        </is>
+      </c>
+      <c r="I52" s="2" t="inlineStr">
+        <is>
+          <t>Merger/Acquisition: News in Focus Browse News Releases All News Releases All Public Company English-only News Releases Overview Multimedia Gallery All Multimedia All Photos All Videos Multimedia Gallery Overview Trending Topics All Trending Topics Business &amp; Money Auto &amp; Transportation All Automo...</t>
+        </is>
+      </c>
+      <c r="J52" s="3" t="inlineStr">
+        <is>
+          <t>https://www.prnewswire.com/news-releases/five9-set-to-join-sp-smallcap-600-302838329.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="inlineStr">
+        <is>
+          <t>S&amp;P 600</t>
+        </is>
+      </c>
+      <c r="B53" s="2" t="inlineStr">
+        <is>
+          <t>Leggett &amp; Platt</t>
+        </is>
+      </c>
+      <c r="C53" s="2" t="inlineStr">
+        <is>
+          <t>LEG</t>
+        </is>
+      </c>
+      <c r="D53" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="E53" s="2" t="inlineStr"/>
+      <c r="F53" s="2" t="inlineStr"/>
+      <c r="G53" s="2" t="inlineStr"/>
+      <c r="H53" s="2" t="inlineStr">
+        <is>
+          <t>Removed, no matching addition found</t>
+        </is>
+      </c>
+      <c r="I53" s="2" t="inlineStr">
+        <is>
           <t>Merger/Acquisition: (NYSE: SGI ) is acquiring Leggett &amp; Platt in a deal expected to be completed soon, pending final closing conditions.</t>
         </is>
       </c>
-      <c r="J51" s="3" t="inlineStr">
+      <c r="J53" s="3" t="inlineStr">
         <is>
           <t>https://www.prnewswire.com/news-releases/tenable-holdings-set-to-join-sp-smallcap-600-302861023.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>S&amp;P 600</t>
+        </is>
+      </c>
+      <c r="B54" s="2" t="inlineStr">
+        <is>
+          <t>Qorvo</t>
+        </is>
+      </c>
+      <c r="C54" s="2" t="inlineStr">
+        <is>
+          <t>QRVO</t>
+        </is>
+      </c>
+      <c r="D54" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="E54" s="2" t="inlineStr"/>
+      <c r="F54" s="2" t="inlineStr"/>
+      <c r="G54" s="2" t="inlineStr"/>
+      <c r="H54" s="2" t="inlineStr">
+        <is>
+          <t>Removed, no matching addition found</t>
+        </is>
+      </c>
+      <c r="I54" s="2" t="inlineStr">
+        <is>
+          <t>Merger/Acquisition: (NASD: SWKS) is acquiring Qorvo in a deal expected to be completed soon, pending final closing conditions.</t>
+        </is>
+      </c>
+      <c r="J54" s="3" t="inlineStr">
+        <is>
+          <t>https://www.prnewswire.com/news-releases/vylor-added-to-the-sp-500-twilio-set-to-join-sp-500-others-to-join-sp-midcap-400-and-sp-smallcap-600-302896675.html</t>
         </is>
       </c>
     </row>
@@ -3001,6 +3145,9 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J49" r:id="rId48"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J50" r:id="rId49"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J51" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J52" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J53" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J54" r:id="rId53"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
🔄 Index Monitor Update - 2026-10-06 03:15:18 UTC
Detected 7 going-forward index changes

Automated commit by GitHub Actions
</commit_message>
<xml_diff>
--- a/index_changes_evidence.xlsx
+++ b/index_changes_evidence.xlsx
@@ -438,7 +438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J54"/>
+  <dimension ref="A1:J55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -3090,6 +3090,46 @@
       <c r="J54" s="3" t="inlineStr">
         <is>
           <t>https://www.prnewswire.com/news-releases/vylor-added-to-the-sp-500-twilio-set-to-join-sp-500-others-to-join-sp-midcap-400-and-sp-smallcap-600-302896675.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="inlineStr">
+        <is>
+          <t>S&amp;P 600</t>
+        </is>
+      </c>
+      <c r="B55" s="2" t="inlineStr">
+        <is>
+          <t>BioLife Solutions</t>
+        </is>
+      </c>
+      <c r="C55" s="2" t="inlineStr">
+        <is>
+          <t>BLFS</t>
+        </is>
+      </c>
+      <c r="D55" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="E55" s="2" t="inlineStr"/>
+      <c r="F55" s="2" t="inlineStr"/>
+      <c r="G55" s="2" t="inlineStr"/>
+      <c r="H55" s="2" t="inlineStr">
+        <is>
+          <t>Removed, no matching addition found</t>
+        </is>
+      </c>
+      <c r="I55" s="2" t="inlineStr">
+        <is>
+          <t>Merger/Acquisition: (NASD:RGEN) is acquiring BioLife Solutions in a deal expected to be completed soon, pending final closing conditions.</t>
+        </is>
+      </c>
+      <c r="J55" s="3" t="inlineStr">
+        <is>
+          <t>https://www.prnewswire.com/news-releases/freshworks-set-to-join-sp-smallcap-600-302899001.html</t>
         </is>
       </c>
     </row>
@@ -3148,6 +3188,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J52" r:id="rId51"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J53" r:id="rId52"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J54" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J55" r:id="rId54"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
🔄 Index Monitor Update - 2026-10-23 06:56:19 UTC
Detected 2 going-forward index changes

Automated commit by GitHub Actions
</commit_message>
<xml_diff>
--- a/index_changes_evidence.xlsx
+++ b/index_changes_evidence.xlsx
@@ -438,7 +438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J55"/>
+  <dimension ref="A1:J56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -3130,6 +3130,46 @@
       <c r="J55" s="3" t="inlineStr">
         <is>
           <t>https://www.prnewswire.com/news-releases/freshworks-set-to-join-sp-smallcap-600-302899001.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>S&amp;P 600</t>
+        </is>
+      </c>
+      <c r="B56" s="2" t="inlineStr">
+        <is>
+          <t>Supernus Pharmaceuticals</t>
+        </is>
+      </c>
+      <c r="C56" s="2" t="inlineStr">
+        <is>
+          <t>SUPN</t>
+        </is>
+      </c>
+      <c r="D56" s="2" t="inlineStr">
+        <is>
+          <t>2026-11-02</t>
+        </is>
+      </c>
+      <c r="E56" s="2" t="inlineStr"/>
+      <c r="F56" s="2" t="inlineStr"/>
+      <c r="G56" s="2" t="inlineStr"/>
+      <c r="H56" s="2" t="inlineStr">
+        <is>
+          <t>Removed, no matching addition found</t>
+        </is>
+      </c>
+      <c r="I56" s="2" t="inlineStr">
+        <is>
+          <t>Merger/Acquisition: (NASD: INDV) is acquiring Supernus Pharmaceuticals in a deal expected to be completed soon, pending final closing conditions.</t>
+        </is>
+      </c>
+      <c r="J56" s="3" t="inlineStr">
+        <is>
+          <t>https://www.prnewswire.com/news-releases/msg-rangers-and-huron-consulting-group-set-to-join-sp-smallcap-600-302917492.html</t>
         </is>
       </c>
     </row>
@@ -3189,6 +3229,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J53" r:id="rId52"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J54" r:id="rId53"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J55" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J56" r:id="rId55"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
🔄 Index Monitor Update - 2026-10-24 06:51:45 UTC
Detected 3 going-forward index changes

Automated commit by GitHub Actions
</commit_message>
<xml_diff>
--- a/index_changes_evidence.xlsx
+++ b/index_changes_evidence.xlsx
@@ -438,7 +438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J56"/>
+  <dimension ref="A1:J57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -3141,17 +3141,17 @@
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>Supernus Pharmaceuticals</t>
+          <t>Arcosa</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>SUPN</t>
+          <t>ACA</t>
         </is>
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>2026-11-02</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="E56" s="2" t="inlineStr"/>
@@ -3164,10 +3164,50 @@
       </c>
       <c r="I56" s="2" t="inlineStr">
         <is>
+          <t>Merger/Acquisition: S&amp;P 500 constituent CRH plc (NYSE: CRH ) has acquired Arcosa in a deal that closed today, October 23.</t>
+        </is>
+      </c>
+      <c r="J56" s="3" t="inlineStr">
+        <is>
+          <t>https://www.prnewswire.com/news-releases/howard-hughes-holdings-set-to-join-sp-smallcap-600-302918511.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="inlineStr">
+        <is>
+          <t>S&amp;P 600</t>
+        </is>
+      </c>
+      <c r="B57" s="2" t="inlineStr">
+        <is>
+          <t>Supernus Pharmaceuticals</t>
+        </is>
+      </c>
+      <c r="C57" s="2" t="inlineStr">
+        <is>
+          <t>SUPN</t>
+        </is>
+      </c>
+      <c r="D57" s="2" t="inlineStr">
+        <is>
+          <t>2026-11-02</t>
+        </is>
+      </c>
+      <c r="E57" s="2" t="inlineStr"/>
+      <c r="F57" s="2" t="inlineStr"/>
+      <c r="G57" s="2" t="inlineStr"/>
+      <c r="H57" s="2" t="inlineStr">
+        <is>
+          <t>Removed, no matching addition found</t>
+        </is>
+      </c>
+      <c r="I57" s="2" t="inlineStr">
+        <is>
           <t>Merger/Acquisition: (NASD: INDV) is acquiring Supernus Pharmaceuticals in a deal expected to be completed soon, pending final closing conditions.</t>
         </is>
       </c>
-      <c r="J56" s="3" t="inlineStr">
+      <c r="J57" s="3" t="inlineStr">
         <is>
           <t>https://www.prnewswire.com/news-releases/msg-rangers-and-huron-consulting-group-set-to-join-sp-smallcap-600-302917492.html</t>
         </is>
@@ -3230,6 +3270,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J54" r:id="rId53"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J55" r:id="rId54"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J56" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J57" r:id="rId56"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
🔄 Index Monitor Update - 2026-10-29 07:59:48 UTC
Detected 3 going-forward index changes

Automated commit by GitHub Actions
</commit_message>
<xml_diff>
--- a/index_changes_evidence.xlsx
+++ b/index_changes_evidence.xlsx
@@ -438,7 +438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J57"/>
+  <dimension ref="A1:J58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -3210,6 +3210,46 @@
       <c r="J57" s="3" t="inlineStr">
         <is>
           <t>https://www.prnewswire.com/news-releases/msg-rangers-and-huron-consulting-group-set-to-join-sp-smallcap-600-302917492.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="inlineStr">
+        <is>
+          <t>S&amp;P 600</t>
+        </is>
+      </c>
+      <c r="B58" s="2" t="inlineStr">
+        <is>
+          <t>Supernus Pharmaceuticals</t>
+        </is>
+      </c>
+      <c r="C58" s="2" t="inlineStr">
+        <is>
+          <t>SUPN</t>
+        </is>
+      </c>
+      <c r="D58" s="2" t="inlineStr">
+        <is>
+          <t>2026-11-03</t>
+        </is>
+      </c>
+      <c r="E58" s="2" t="inlineStr"/>
+      <c r="F58" s="2" t="inlineStr"/>
+      <c r="G58" s="2" t="inlineStr"/>
+      <c r="H58" s="2" t="inlineStr">
+        <is>
+          <t>Removed, no matching addition found</t>
+        </is>
+      </c>
+      <c r="I58" s="2" t="inlineStr">
+        <is>
+          <t>Merger/Acquisition: (NASD: INDV) is acquiring Supernus Pharmaceuticals in a transaction expected to close soon, subject to final closing conditions.</t>
+        </is>
+      </c>
+      <c r="J58" s="3" t="inlineStr">
+        <is>
+          <t>https://www.prnewswire.com/news-releases/updated-effective-date-huron-consulting-group-set-to-join-sp-smallcap-600-302922778.html</t>
         </is>
       </c>
     </row>
@@ -3271,6 +3311,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J55" r:id="rId54"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J56" r:id="rId55"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J57" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J58" r:id="rId57"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
🔄 Index Monitor Update - 2026-10-31 07:58:32 UTC
Detected 7 going-forward index changes

Automated commit by GitHub Actions
</commit_message>
<xml_diff>
--- a/index_changes_evidence.xlsx
+++ b/index_changes_evidence.xlsx
@@ -438,7 +438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J58"/>
+  <dimension ref="A1:J60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1360,52 +1360,40 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>S&amp;P 600</t>
+          <t>S&amp;P 500</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Brandywine Realty Trust</t>
+          <t>Kenvue</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>BDN</t>
+          <t>KVUE</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
-        </is>
-      </c>
-      <c r="E20" s="2" t="inlineStr">
-        <is>
-          <t>Versant Media Group</t>
-        </is>
-      </c>
-      <c r="F20" s="2" t="inlineStr">
-        <is>
-          <t>VSNT</t>
-        </is>
-      </c>
-      <c r="G20" s="2" t="inlineStr">
-        <is>
-          <t>2026-01-07</t>
-        </is>
-      </c>
+          <t>2026-11-04</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr"/>
+      <c r="F20" s="2" t="inlineStr"/>
+      <c r="G20" s="2" t="inlineStr"/>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>Same effective date</t>
+          <t>Removed, no matching addition found</t>
         </is>
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>Spin-off: VSNT was spun off fromComcastand replaced BDN which was no longer representative of the small-cap market space.[38]</t>
+          <t>Merger/Acquisition: S&amp;P 500 constituent Kimberly-Clark (NASD: KMB) is acquiring Kenvue in a deal expected to be completed soon, pending final closing conditions.</t>
         </is>
       </c>
       <c r="J20" s="3" t="inlineStr">
         <is>
-          <t>https://en.wikipedia.org/wiki/List_of_S%26P_600_companies</t>
+          <t>https://www.prnewswire.com/news-releases/okta-set-to-join-sp-500-others-to-join-sp-midcap-400-and-sp-smallcap-600-302925405.html</t>
         </is>
       </c>
     </row>
@@ -1417,32 +1405,32 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Guess, Inc.</t>
+          <t>Brandywine Realty Trust</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>GES</t>
+          <t>BDN</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>2026-01-26</t>
+          <t>2026-01-07</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>Winmark</t>
+          <t>Versant Media Group</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>WINA</t>
+          <t>VSNT</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>2026-01-26</t>
+          <t>2026-01-07</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
@@ -1452,7 +1440,7 @@
       </c>
       <c r="I21" s="2" t="inlineStr">
         <is>
-          <t>Merger/Acquisition: WINA replaced GES after it was acquired byAuthentic Brands Groupand the Rolling Stockholders.[37]</t>
+          <t>Spin-off: VSNT was spun off fromComcastand replaced BDN which was no longer representative of the small-cap market space.[38]</t>
         </is>
       </c>
       <c r="J21" s="3" t="inlineStr">
@@ -1469,32 +1457,32 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>TTM Technologies</t>
+          <t>Guess, Inc.</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>TTMI</t>
+          <t>GES</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>2026-01-30</t>
+          <t>2026-01-26</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>Amneal Pharmaceuticals</t>
+          <t>Winmark</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>AMRX</t>
+          <t>WINA</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>2026-01-30</t>
+          <t>2026-01-26</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
@@ -1504,7 +1492,7 @@
       </c>
       <c r="I22" s="2" t="inlineStr">
         <is>
-          <t>Merger/Acquisition: AMRX replaced TTMI, which replaced Civitas Resources in theS&amp;P 400after it was acquired bySM Energy.[36]</t>
+          <t>Merger/Acquisition: WINA replaced GES after it was acquired byAuthentic Brands Groupand the Rolling Stockholders.[37]</t>
         </is>
       </c>
       <c r="J22" s="3" t="inlineStr">
@@ -1521,32 +1509,32 @@
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>Advanced Energy</t>
+          <t>TTM Technologies</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>AEIS</t>
+          <t>TTMI</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>2026-02-02</t>
+          <t>2026-01-30</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>Apellis Pharmaceuticals</t>
+          <t>Amneal Pharmaceuticals</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>APLS</t>
+          <t>AMRX</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>2026-02-02</t>
+          <t>2026-01-30</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
@@ -1556,7 +1544,7 @@
       </c>
       <c r="I23" s="2" t="inlineStr">
         <is>
-          <t>Merger/Acquisition: APLS replaced AEIS, which replacedComericain the S&amp;P 400 after it was acquired byFifth Third Bank.[36]</t>
+          <t>Merger/Acquisition: AMRX replaced TTMI, which replaced Civitas Resources in theS&amp;P 400after it was acquired bySM Energy.[36]</t>
         </is>
       </c>
       <c r="J23" s="3" t="inlineStr">
@@ -1573,32 +1561,32 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>Dynavax Technologies</t>
+          <t>Advanced Energy</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>DVAX</t>
+          <t>AEIS</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>2026-02-10</t>
+          <t>2026-02-02</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>OneSpaWorld Holdings</t>
+          <t>Apellis Pharmaceuticals</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>OSW</t>
+          <t>APLS</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>2026-02-10</t>
+          <t>2026-02-02</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr">
@@ -1608,7 +1596,7 @@
       </c>
       <c r="I24" s="2" t="inlineStr">
         <is>
-          <t>Merger/Acquisition: OSW replaced DVAX after it was acquired bySanofi.[35]</t>
+          <t>Merger/Acquisition: APLS replaced AEIS, which replacedComericain the S&amp;P 400 after it was acquired byFifth Third Bank.[36]</t>
         </is>
       </c>
       <c r="J24" s="3" t="inlineStr">
@@ -1625,32 +1613,32 @@
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>TreeHouse Foods</t>
+          <t>Dynavax Technologies</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>THS</t>
+          <t>DVAX</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>2026-02-11</t>
+          <t>2026-02-10</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>Merchants Bancorp</t>
+          <t>OneSpaWorld Holdings</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>MBIN</t>
+          <t>OSW</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>2026-02-11</t>
+          <t>2026-02-10</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
@@ -1660,7 +1648,7 @@
       </c>
       <c r="I25" s="2" t="inlineStr">
         <is>
-          <t>Merger/Acquisition: MBIN replaced THS after it was acquired by Investindustrial S.A.[34]</t>
+          <t>Merger/Acquisition: OSW replaced DVAX after it was acquired bySanofi.[35]</t>
         </is>
       </c>
       <c r="J25" s="3" t="inlineStr">
@@ -1677,32 +1665,32 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>Hillenbrand</t>
+          <t>TreeHouse Foods</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>HI</t>
+          <t>THS</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>2026-02-12</t>
+          <t>2026-02-11</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>RingCentral</t>
+          <t>Merchants Bancorp</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>RNG</t>
+          <t>MBIN</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>2026-02-12</t>
+          <t>2026-02-11</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr">
@@ -1712,7 +1700,7 @@
       </c>
       <c r="I26" s="2" t="inlineStr">
         <is>
-          <t>Merger/Acquisition: RNG replaced HI after it was acquired byLone Star Funds.[33]</t>
+          <t>Merger/Acquisition: MBIN replaced THS after it was acquired by Investindustrial S.A.[34]</t>
         </is>
       </c>
       <c r="J26" s="3" t="inlineStr">
@@ -1729,32 +1717,32 @@
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>Alexander &amp; Baldwin</t>
+          <t>Hillenbrand</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>ALEX</t>
+          <t>HI</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>2026-03-13</t>
+          <t>2026-02-12</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>Napco Security Technologies</t>
+          <t>RingCentral</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>NSSC</t>
+          <t>RNG</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>2026-03-13</t>
+          <t>2026-02-12</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr">
@@ -1764,7 +1752,7 @@
       </c>
       <c r="I27" s="2" t="inlineStr">
         <is>
-          <t>Merger/Acquisition: NSSC replaced ALEX after it was acquired by an investor group comprising MW Group and funds affiliated with DivcoWest andBlackstone Real Estate.[32]</t>
+          <t>Merger/Acquisition: RNG replaced HI after it was acquired byLone Star Funds.[33]</t>
         </is>
       </c>
       <c r="J27" s="3" t="inlineStr">
@@ -1781,32 +1769,32 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>Tegna Inc.</t>
+          <t>Alexander &amp; Baldwin</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>TGNA</t>
+          <t>ALEX</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-13</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>Vita Coco</t>
+          <t>Napco Security Technologies</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>COCO</t>
+          <t>NSSC</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-13</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr">
@@ -1816,7 +1804,7 @@
       </c>
       <c r="I28" s="2" t="inlineStr">
         <is>
-          <t>Merger/Acquisition: COCO replaced TGNA after it was acquired byNexstar Media Group.[31]</t>
+          <t>Merger/Acquisition: NSSC replaced ALEX after it was acquired by an investor group comprising MW Group and funds affiliated with DivcoWest andBlackstone Real Estate.[32]</t>
         </is>
       </c>
       <c r="J28" s="3" t="inlineStr">
@@ -1833,32 +1821,32 @@
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>Titan International, Inc.</t>
+          <t>Tegna Inc.</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>TWI</t>
+          <t>TGNA</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>Versigent</t>
+          <t>Vita Coco</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>VGNT</t>
+          <t>COCO</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -1868,7 +1856,7 @@
       </c>
       <c r="I29" s="2" t="inlineStr">
         <is>
-          <t>Spin-off: VGNT was spun off fromAptivand replaced TWI which was no longer representative of the small-cap market space.[30]</t>
+          <t>Merger/Acquisition: COCO replaced TGNA after it was acquired byNexstar Media Group.[31]</t>
         </is>
       </c>
       <c r="J29" s="3" t="inlineStr">
@@ -1885,32 +1873,32 @@
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>Air Lease Corporation</t>
+          <t>Titan International, Inc.</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>AL</t>
+          <t>TWI</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-04-02</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>Atmus Filtration Technologies</t>
+          <t>Versigent</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>ATMU</t>
+          <t>VGNT</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-04-02</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -1920,7 +1908,7 @@
       </c>
       <c r="I30" s="2" t="inlineStr">
         <is>
-          <t>Merger/Acquisition: ATMU replaced AL after it was acquired bySumitomo Corporation.[29]</t>
+          <t>Spin-off: VGNT was spun off fromAptivand replaced TWI which was no longer representative of the small-cap market space.[30]</t>
         </is>
       </c>
       <c r="J30" s="3" t="inlineStr">
@@ -1937,32 +1925,32 @@
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>Sealed Air</t>
+          <t>Air Lease Corporation</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>SEE</t>
+          <t>AL</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>Diebold Nixdorf</t>
+          <t>Atmus Filtration Technologies</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>DBD</t>
+          <t>ATMU</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr">
@@ -1972,7 +1960,7 @@
       </c>
       <c r="I31" s="2" t="inlineStr">
         <is>
-          <t>Merger/Acquisition: DBD replaced SEE after it was acquired byClayton, Dubilier &amp; Rice.[27]</t>
+          <t>Merger/Acquisition: ATMU replaced AL after it was acquired bySumitomo Corporation.[29]</t>
         </is>
       </c>
       <c r="J31" s="3" t="inlineStr">
@@ -1989,32 +1977,32 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>Golden Entertainment</t>
+          <t>Sealed Air</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>GDEN</t>
+          <t>SEE</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>Lifestance Health</t>
+          <t>Diebold Nixdorf</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>LFST</t>
+          <t>DBD</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr">
@@ -2024,7 +2012,7 @@
       </c>
       <c r="I32" s="2" t="inlineStr">
         <is>
-          <t>Merger/Acquisition: LFST replaced GDEN after it was acquired byVici PropertiesandBlake L. Sartini.[25]</t>
+          <t>Merger/Acquisition: DBD replaced SEE after it was acquired byClayton, Dubilier &amp; Rice.[27]</t>
         </is>
       </c>
       <c r="J32" s="3" t="inlineStr">
@@ -2041,32 +2029,32 @@
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>Apellis Pharmaceuticals</t>
+          <t>Golden Entertainment</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>APLS</t>
+          <t>GDEN</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>Alignment Healthcare</t>
+          <t>Lifestance Health</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>ALHC</t>
+          <t>LFST</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="H33" s="2" t="inlineStr">
@@ -2076,7 +2064,7 @@
       </c>
       <c r="I33" s="2" t="inlineStr">
         <is>
-          <t>Merger/Acquisition: ALHC replaced SNCY after it was acquired byAllegiant Travel Company.[22] | Merger/Acquisition: RELY replaced APLS after it was acquired byBiogen.[23]</t>
+          <t>Merger/Acquisition: LFST replaced GDEN after it was acquired byVici PropertiesandBlake L. Sartini.[25]</t>
         </is>
       </c>
       <c r="J33" s="3" t="inlineStr">
@@ -2093,12 +2081,12 @@
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>Sun Country Airlines</t>
+          <t>Apellis Pharmaceuticals</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>SNCY</t>
+          <t>APLS</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
@@ -2108,12 +2096,12 @@
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>Bright Horizons</t>
+          <t>Alignment Healthcare</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>BFAM</t>
+          <t>ALHC</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
@@ -2128,7 +2116,7 @@
       </c>
       <c r="I34" s="2" t="inlineStr">
         <is>
-          <t>Merger/Acquisition: BFAM replaced TPH after it was acquired bySumitomo Forestry.[23] | Merger/Acquisition: ALHC replaced SNCY after it was acquired byAllegiant Travel Company.[22]</t>
+          <t>Merger/Acquisition: ALHC replaced SNCY after it was acquired byAllegiant Travel Company.[22] | Merger/Acquisition: RELY replaced APLS after it was acquired byBiogen.[23]</t>
         </is>
       </c>
       <c r="J34" s="3" t="inlineStr">
@@ -2145,12 +2133,12 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>Tri Pointe Homes</t>
+          <t>Sun Country Airlines</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>TPH</t>
+          <t>SNCY</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
@@ -2160,12 +2148,12 @@
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>Remitly</t>
+          <t>Bright Horizons</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>RELY</t>
+          <t>BFAM</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
@@ -2180,7 +2168,7 @@
       </c>
       <c r="I35" s="2" t="inlineStr">
         <is>
-          <t>Merger/Acquisition: RELY replaced APLS after it was acquired byBiogen.[23] | Merger/Acquisition: BFAM replaced TPH after it was acquired bySumitomo Forestry.[23]</t>
+          <t>Merger/Acquisition: BFAM replaced TPH after it was acquired bySumitomo Forestry.[23] | Merger/Acquisition: ALHC replaced SNCY after it was acquired byAllegiant Travel Company.[22]</t>
         </is>
       </c>
       <c r="J35" s="3" t="inlineStr">
@@ -2197,32 +2185,32 @@
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>CSG Systems</t>
+          <t>Tri Pointe Homes</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>CSGS</t>
+          <t>TPH</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>Flowers Foods</t>
+          <t>Remitly</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>FLO</t>
+          <t>RELY</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr">
@@ -2232,7 +2220,7 @@
       </c>
       <c r="I36" s="2" t="inlineStr">
         <is>
-          <t>Merger/Acquisition: FLO replaced CSGS after it was acquired byNEC.[21]</t>
+          <t>Merger/Acquisition: RELY replaced APLS after it was acquired byBiogen.[23] | Merger/Acquisition: BFAM replaced TPH after it was acquired bySumitomo Forestry.[23]</t>
         </is>
       </c>
       <c r="J36" s="3" t="inlineStr">
@@ -2249,12 +2237,12 @@
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>Enviri</t>
+          <t>CSG Systems</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>NVRI</t>
+          <t>CSGS</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
@@ -2264,12 +2252,12 @@
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>Peloton Interactive</t>
+          <t>Flowers Foods</t>
         </is>
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>PTON</t>
+          <t>FLO</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
@@ -2284,7 +2272,7 @@
       </c>
       <c r="I37" s="2" t="inlineStr">
         <is>
-          <t>Spin-off: PTON replaced NVRI after it spun off assets into a new publicly traded company. The new publicly traded company was not representative of the small-cap market space.[20]</t>
+          <t>Merger/Acquisition: FLO replaced CSGS after it was acquired byNEC.[21]</t>
         </is>
       </c>
       <c r="J37" s="3" t="inlineStr">
@@ -2301,32 +2289,32 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>Mister Car Wash</t>
+          <t>Enviri</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>MCW</t>
+          <t>NVRI</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>F&amp;G</t>
+          <t>Peloton Interactive</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>FG</t>
+          <t>PTON</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="H38" s="2" t="inlineStr">
@@ -2336,7 +2324,7 @@
       </c>
       <c r="I38" s="2" t="inlineStr">
         <is>
-          <t>Merger/Acquisition: FG replaced MCW after it was acquired byLeonard Green &amp; Partners.[21]</t>
+          <t>Spin-off: PTON replaced NVRI after it spun off assets into a new publicly traded company. The new publicly traded company was not representative of the small-cap market space.[20]</t>
         </is>
       </c>
       <c r="J38" s="3" t="inlineStr">
@@ -2353,32 +2341,32 @@
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>Veris Residential</t>
+          <t>Mister Car Wash</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>VRE</t>
+          <t>MCW</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>Universal Technical Institute</t>
+          <t>F&amp;G</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>UTI</t>
+          <t>FG</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="H39" s="2" t="inlineStr">
@@ -2388,7 +2376,7 @@
       </c>
       <c r="I39" s="2" t="inlineStr">
         <is>
-          <t>Merger/Acquisition: UTI replaced VRE after it was acquired by Affinius Capital and Vista Hill Partners.[20]</t>
+          <t>Merger/Acquisition: FG replaced MCW after it was acquired byLeonard Green &amp; Partners.[21]</t>
         </is>
       </c>
       <c r="J39" s="3" t="inlineStr">
@@ -2405,32 +2393,32 @@
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>American Woodmark</t>
+          <t>Veris Residential</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>AMWD</t>
+          <t>VRE</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>Dave</t>
+          <t>Universal Technical Institute</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>DAVE</t>
+          <t>UTI</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr">
@@ -2440,7 +2428,7 @@
       </c>
       <c r="I40" s="2" t="inlineStr">
         <is>
-          <t>Merger/Acquisition: DAVE replaced AMWD after it was acquired by MasterBrand Inc.[19]</t>
+          <t>Merger/Acquisition: UTI replaced VRE after it was acquired by Affinius Capital and Vista Hill Partners.[20]</t>
         </is>
       </c>
       <c r="J40" s="3" t="inlineStr">
@@ -2457,32 +2445,32 @@
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>Shutterstock</t>
+          <t>American Woodmark</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>SSTK</t>
+          <t>AMWD</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>EPAM Systems</t>
+          <t>Dave</t>
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>EPAM</t>
+          <t>DAVE</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="H41" s="2" t="inlineStr">
@@ -2492,7 +2480,7 @@
       </c>
       <c r="I41" s="2" t="inlineStr">
         <is>
-          <t>Merger/Acquisition: EPAM was moved from theS&amp;P 500as it was more representative of the small cap market space. SSTK was removed from theS&amp;P 600as it was merged withGetty Images.[19]</t>
+          <t>Merger/Acquisition: DAVE replaced AMWD after it was acquired by MasterBrand Inc.[19]</t>
         </is>
       </c>
       <c r="J41" s="3" t="inlineStr">
@@ -2509,32 +2497,32 @@
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>Core Laboratories</t>
+          <t>Shutterstock</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>CLB</t>
+          <t>SSTK</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>Mobility Global</t>
+          <t>EPAM Systems</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>MBGL</t>
+          <t>EPAM</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr">
@@ -2544,7 +2532,7 @@
       </c>
       <c r="I42" s="2" t="inlineStr">
         <is>
-          <t>Spin-off: MBGL was spun off fromS&amp;P Globaland replaced CLB which was no longer representative of the small-cap market space.[13]</t>
+          <t>Merger/Acquisition: EPAM was moved from theS&amp;P 500as it was more representative of the small cap market space. SSTK was removed from theS&amp;P 600as it was merged withGetty Images.[19]</t>
         </is>
       </c>
       <c r="J42" s="3" t="inlineStr">
@@ -2561,32 +2549,32 @@
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>Whitestone REIT</t>
+          <t>Core Laboratories</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>WSR</t>
+          <t>CLB</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>Centrus Energy</t>
+          <t>Mobility Global</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>LEU</t>
+          <t>MBGL</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="H43" s="2" t="inlineStr">
@@ -2596,7 +2584,7 @@
       </c>
       <c r="I43" s="2" t="inlineStr">
         <is>
-          <t>Merger/Acquisition: LEU replaced WSR after it was acquired byAres Management.[11]</t>
+          <t>Spin-off: MBGL was spun off fromS&amp;P Globaland replaced CLB which was no longer representative of the small-cap market space.[13]</t>
         </is>
       </c>
       <c r="J43" s="3" t="inlineStr">
@@ -2613,32 +2601,32 @@
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>Hertz Global Holdings</t>
+          <t>Whitestone REIT</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>HTZ</t>
+          <t>WSR</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>ADI Global Distribution</t>
+          <t>Centrus Energy</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>ADIG</t>
+          <t>LEU</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="H44" s="2" t="inlineStr">
@@ -2648,12 +2636,12 @@
       </c>
       <c r="I44" s="2" t="inlineStr">
         <is>
-          <t>Merger/Acquisition: News in Focus Browse News Releases All News Releases All Public Company English-only News Releases Overview Multimedia Gallery All Multimedia All Photos All Videos Multimedia Gallery Overview Trending Topics All Trending Topics Business &amp; Money Auto &amp; Transportation All Automo... | Spin-off: ADIG was spun off fromResideoand replaced HTZ which was no longer representative of the small-cap market space.[5]</t>
+          <t>Merger/Acquisition: LEU replaced WSR after it was acquired byAres Management.[11]</t>
         </is>
       </c>
       <c r="J44" s="3" t="inlineStr">
         <is>
-          <t>https://www.prnewswire.com/news-releases/ferguson-enterprises-set-to-join-sp-500-and-adi-global-distribution-to-join-sp-smallcap-600-302840407.html</t>
+          <t>https://en.wikipedia.org/wiki/List_of_S%26P_600_companies</t>
         </is>
       </c>
     </row>
@@ -2665,47 +2653,47 @@
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>Kennedy-Wilson Holdings</t>
+          <t>Hertz Global Holdings</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>KW</t>
+          <t>HTZ</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>National Health Investors</t>
+          <t>ADI Global Distribution</t>
         </is>
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>NHI</t>
+          <t>ADIG</t>
         </is>
       </c>
       <c r="G45" s="2" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="H45" s="2" t="inlineStr">
         <is>
-          <t>Different effective dates — paired for reference only</t>
+          <t>Same effective date</t>
         </is>
       </c>
       <c r="I45" s="2" t="inlineStr">
         <is>
-          <t>Merger/Acquisition: News in Focus Browse News Releases All News Releases All Public Company English-only News Releases Overview Multimedia Gallery All Multimedia All Photos All Videos Multimedia Gallery Overview Trending Topics All Trending Topics Business &amp; Money Auto &amp; Transportation All Automo... | Merger/Acquisition: A consortium led by KW's CEO with Fairfax Financial Holdings Limited (TSE: FFH) is acquiring Kennedy-Wilson Holdings in a deal expected to close soon, pending final closing conditions.</t>
+          <t>Merger/Acquisition: News in Focus Browse News Releases All News Releases All Public Company English-only News Releases Overview Multimedia Gallery All Multimedia All Photos All Videos Multimedia Gallery Overview Trending Topics All Trending Topics Business &amp; Money Auto &amp; Transportation All Automo... | Spin-off: ADIG was spun off fromResideoand replaced HTZ which was no longer representative of the small-cap market space.[5]</t>
         </is>
       </c>
       <c r="J45" s="3" t="inlineStr">
         <is>
-          <t>https://www.prnewswire.com/news-releases/honeywell-aerospace-set-to-join-sp-500--sp-100-others-to-join-sp-midcap-400-and-sp-smallcap-600-302808386.html</t>
+          <t>https://www.prnewswire.com/news-releases/ferguson-enterprises-set-to-join-sp-500-and-adi-global-distribution-to-join-sp-smallcap-600-302840407.html</t>
         </is>
       </c>
     </row>
@@ -2717,32 +2705,32 @@
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>ProAssurance</t>
+          <t>Kennedy-Wilson Holdings</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>PRA</t>
+          <t>KW</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>Construction Partners</t>
+          <t>National Health Investors</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>ROAD</t>
+          <t>NHI</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="H46" s="2" t="inlineStr">
@@ -2752,12 +2740,12 @@
       </c>
       <c r="I46" s="2" t="inlineStr">
         <is>
-          <t>Merger/Acquisition: News in Focus Browse News Releases All News Releases All Public Company English-only News Releases Overview Multimedia Gallery All Multimedia All Photos All Videos Multimedia Gallery Overview Trending Topics All Trending Topics Business &amp; Money Auto &amp; Transportation All Automo... | Merger/Acquisition: The Doctors Company is acquiring ProAssurance in a cash deal expected to close soon, pending final closing conditions.</t>
+          <t>Merger/Acquisition: News in Focus Browse News Releases All News Releases All Public Company English-only News Releases Overview Multimedia Gallery All Multimedia All Photos All Videos Multimedia Gallery Overview Trending Topics All Trending Topics Business &amp; Money Auto &amp; Transportation All Automo... | Merger/Acquisition: A consortium led by KW's CEO with Fairfax Financial Holdings Limited (TSE: FFH) is acquiring Kennedy-Wilson Holdings in a deal expected to close soon, pending final closing conditions.</t>
         </is>
       </c>
       <c r="J46" s="3" t="inlineStr">
         <is>
-          <t>https://www.prnewswire.com/news-releases/molina-healthcare-set-to-join-sp-midcap-400-and-construction-partners-to-join-sp-smallcap-600-302828046.html</t>
+          <t>https://www.prnewswire.com/news-releases/honeywell-aerospace-set-to-join-sp-500--sp-100-others-to-join-sp-midcap-400-and-sp-smallcap-600-302808386.html</t>
         </is>
       </c>
     </row>
@@ -2769,32 +2757,32 @@
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>Select Medical Holdings</t>
+          <t>ProAssurance</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>SEM</t>
+          <t>PRA</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>The Trade Desk</t>
+          <t>Construction Partners</t>
         </is>
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>TTD</t>
+          <t>ROAD</t>
         </is>
       </c>
       <c r="G47" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="H47" s="2" t="inlineStr">
@@ -2804,12 +2792,12 @@
       </c>
       <c r="I47" s="2" t="inlineStr">
         <is>
-          <t>Merger/Acquisition: News in Focus Browse News Releases All News Releases All Public Company English-only News Releases Overview Multimedia Gallery All Multimedia All Photos All Videos Multimedia Gallery Overview Trending Topics All Trending Topics Business &amp; Money Auto &amp; Transportation All Automo... | Merger/Acquisition: Select Medical Holdings is being acquired in a deal expected to be completed soon, pending final closing conditions.</t>
+          <t>Merger/Acquisition: News in Focus Browse News Releases All News Releases All Public Company English-only News Releases Overview Multimedia Gallery All Multimedia All Photos All Videos Multimedia Gallery Overview Trending Topics All Trending Topics Business &amp; Money Auto &amp; Transportation All Automo... | Merger/Acquisition: The Doctors Company is acquiring ProAssurance in a cash deal expected to close soon, pending final closing conditions.</t>
         </is>
       </c>
       <c r="J47" s="3" t="inlineStr">
         <is>
-          <t>https://www.prnewswire.com/news-releases/bloom-energy-illumina-and-everpure-set-to-join-sp-500-others-to-join-sp-100-sp-midcap-400-and-sp-smallcap-600-302870517.html</t>
+          <t>https://www.prnewswire.com/news-releases/molina-healthcare-set-to-join-sp-midcap-400-and-construction-partners-to-join-sp-smallcap-600-302828046.html</t>
         </is>
       </c>
     </row>
@@ -2821,35 +2809,47 @@
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>Stellar Bancorp</t>
+          <t>Select Medical Holdings</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>STEL</t>
+          <t>SEM</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
-        </is>
-      </c>
-      <c r="E48" s="2" t="inlineStr"/>
-      <c r="F48" s="2" t="inlineStr"/>
-      <c r="G48" s="2" t="inlineStr"/>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="E48" s="2" t="inlineStr">
+        <is>
+          <t>The Trade Desk</t>
+        </is>
+      </c>
+      <c r="F48" s="2" t="inlineStr">
+        <is>
+          <t>TTD</t>
+        </is>
+      </c>
+      <c r="G48" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
       <c r="H48" s="2" t="inlineStr">
         <is>
-          <t>Removed, no matching addition found</t>
+          <t>Different effective dates — paired for reference only</t>
         </is>
       </c>
       <c r="I48" s="2" t="inlineStr">
         <is>
-          <t>Merger/Acquisition: (NYSE: PB ) is acquiring Stellar Bancorp in a deal expected to close July 1.</t>
+          <t>Merger/Acquisition: News in Focus Browse News Releases All News Releases All Public Company English-only News Releases Overview Multimedia Gallery All Multimedia All Photos All Videos Multimedia Gallery Overview Trending Topics All Trending Topics Business &amp; Money Auto &amp; Transportation All Automo... | Merger/Acquisition: Select Medical Holdings is being acquired in a deal expected to be completed soon, pending final closing conditions.</t>
         </is>
       </c>
       <c r="J48" s="3" t="inlineStr">
         <is>
-          <t>https://www.prnewswire.com/news-releases/allison-transmission-holdings-set-to-join-sp-midcap-400-and-goodyear-tire--rubber-to-join-sp-smallcap-600-302815143.html</t>
+          <t>https://www.prnewswire.com/news-releases/bloom-energy-illumina-and-everpure-set-to-join-sp-500-others-to-join-sp-100-sp-midcap-400-and-sp-smallcap-600-302870517.html</t>
         </is>
       </c>
     </row>
@@ -2861,17 +2861,17 @@
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>Whitestone REIT</t>
+          <t>Stellar Bancorp</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>WSR</t>
+          <t>STEL</t>
         </is>
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="E49" s="2" t="inlineStr"/>
@@ -2884,12 +2884,12 @@
       </c>
       <c r="I49" s="2" t="inlineStr">
         <is>
-          <t>Merger/Acquisition: (NYSE: ARES ) is acquiring Whitestone REIT in a deal expected to close on or about that date, pending final closing conditions.</t>
+          <t>Merger/Acquisition: (NYSE: PB ) is acquiring Stellar Bancorp in a deal expected to close July 1.</t>
         </is>
       </c>
       <c r="J49" s="3" t="inlineStr">
         <is>
-          <t>https://www.prnewswire.com/news-releases/midera-food-processing-and-centrus-energy-set-to-join-sp-smallcap-600-302817273.html</t>
+          <t>https://www.prnewswire.com/news-releases/allison-transmission-holdings-set-to-join-sp-midcap-400-and-goodyear-tire--rubber-to-join-sp-smallcap-600-302815143.html</t>
         </is>
       </c>
     </row>
@@ -2901,17 +2901,17 @@
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>Catalyst Pharmaceuticals</t>
+          <t>Whitestone REIT</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>CPRX</t>
+          <t>WSR</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="E50" s="2" t="inlineStr"/>
@@ -2924,12 +2924,12 @@
       </c>
       <c r="I50" s="2" t="inlineStr">
         <is>
-          <t>Merger/Acquisition: is acquiring Catalyst Pharmaceuticals in a deal expected to close soon, pending final closing conditions.</t>
+          <t>Merger/Acquisition: (NYSE: ARES ) is acquiring Whitestone REIT in a deal expected to close on or about that date, pending final closing conditions.</t>
         </is>
       </c>
       <c r="J50" s="3" t="inlineStr">
         <is>
-          <t>https://www.prnewswire.com/news-releases/solaris-energy-infrastructure-set-to-join-sp-smallcap-600-302822362.html</t>
+          <t>https://www.prnewswire.com/news-releases/midera-food-processing-and-centrus-energy-set-to-join-sp-smallcap-600-302817273.html</t>
         </is>
       </c>
     </row>
@@ -2941,17 +2941,17 @@
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>Avanos Medical</t>
+          <t>Catalyst Pharmaceuticals</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>AVNS</t>
+          <t>CPRX</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="E51" s="2" t="inlineStr"/>
@@ -2964,12 +2964,12 @@
       </c>
       <c r="I51" s="2" t="inlineStr">
         <is>
-          <t>Merger/Acquisition: American Industrial Partners is acquiring Avanos Medical in a deal expected to close soon, pending final closing conditions.</t>
+          <t>Merger/Acquisition: is acquiring Catalyst Pharmaceuticals in a deal expected to close soon, pending final closing conditions.</t>
         </is>
       </c>
       <c r="J51" s="3" t="inlineStr">
         <is>
-          <t>https://www.prnewswire.com/news-releases/krystal-biotech-set-to-join-sp-midcap-400-tutor-perini-and-v2x-to-join-sp-smallcap-600-302830022.html</t>
+          <t>https://www.prnewswire.com/news-releases/solaris-energy-infrastructure-set-to-join-sp-smallcap-600-302822362.html</t>
         </is>
       </c>
     </row>
@@ -2981,17 +2981,17 @@
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>Two Harbors Investment</t>
+          <t>Avanos Medical</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>TWO</t>
+          <t>AVNS</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="E52" s="2" t="inlineStr"/>
@@ -3004,12 +3004,12 @@
       </c>
       <c r="I52" s="2" t="inlineStr">
         <is>
-          <t>Merger/Acquisition: News in Focus Browse News Releases All News Releases All Public Company English-only News Releases Overview Multimedia Gallery All Multimedia All Photos All Videos Multimedia Gallery Overview Trending Topics All Trending Topics Business &amp; Money Auto &amp; Transportation All Automo...</t>
+          <t>Merger/Acquisition: American Industrial Partners is acquiring Avanos Medical in a deal expected to close soon, pending final closing conditions.</t>
         </is>
       </c>
       <c r="J52" s="3" t="inlineStr">
         <is>
-          <t>https://www.prnewswire.com/news-releases/five9-set-to-join-sp-smallcap-600-302838329.html</t>
+          <t>https://www.prnewswire.com/news-releases/krystal-biotech-set-to-join-sp-midcap-400-tutor-perini-and-v2x-to-join-sp-smallcap-600-302830022.html</t>
         </is>
       </c>
     </row>
@@ -3021,17 +3021,17 @@
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>Leggett &amp; Platt</t>
+          <t>Two Harbors Investment</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>LEG</t>
+          <t>TWO</t>
         </is>
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="E53" s="2" t="inlineStr"/>
@@ -3044,12 +3044,12 @@
       </c>
       <c r="I53" s="2" t="inlineStr">
         <is>
-          <t>Merger/Acquisition: (NYSE: SGI ) is acquiring Leggett &amp; Platt in a deal expected to be completed soon, pending final closing conditions.</t>
+          <t>Merger/Acquisition: News in Focus Browse News Releases All News Releases All Public Company English-only News Releases Overview Multimedia Gallery All Multimedia All Photos All Videos Multimedia Gallery Overview Trending Topics All Trending Topics Business &amp; Money Auto &amp; Transportation All Automo...</t>
         </is>
       </c>
       <c r="J53" s="3" t="inlineStr">
         <is>
-          <t>https://www.prnewswire.com/news-releases/tenable-holdings-set-to-join-sp-smallcap-600-302861023.html</t>
+          <t>https://www.prnewswire.com/news-releases/five9-set-to-join-sp-smallcap-600-302838329.html</t>
         </is>
       </c>
     </row>
@@ -3061,17 +3061,17 @@
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>Qorvo</t>
+          <t>Leggett &amp; Platt</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>QRVO</t>
+          <t>LEG</t>
         </is>
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="E54" s="2" t="inlineStr"/>
@@ -3084,12 +3084,12 @@
       </c>
       <c r="I54" s="2" t="inlineStr">
         <is>
-          <t>Merger/Acquisition: (NASD: SWKS) is acquiring Qorvo in a deal expected to be completed soon, pending final closing conditions.</t>
+          <t>Merger/Acquisition: (NYSE: SGI ) is acquiring Leggett &amp; Platt in a deal expected to be completed soon, pending final closing conditions.</t>
         </is>
       </c>
       <c r="J54" s="3" t="inlineStr">
         <is>
-          <t>https://www.prnewswire.com/news-releases/vylor-added-to-the-sp-500-twilio-set-to-join-sp-500-others-to-join-sp-midcap-400-and-sp-smallcap-600-302896675.html</t>
+          <t>https://www.prnewswire.com/news-releases/tenable-holdings-set-to-join-sp-smallcap-600-302861023.html</t>
         </is>
       </c>
     </row>
@@ -3101,17 +3101,17 @@
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>BioLife Solutions</t>
+          <t>Qorvo</t>
         </is>
       </c>
       <c r="C55" s="2" t="inlineStr">
         <is>
-          <t>BLFS</t>
+          <t>QRVO</t>
         </is>
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="E55" s="2" t="inlineStr"/>
@@ -3124,12 +3124,12 @@
       </c>
       <c r="I55" s="2" t="inlineStr">
         <is>
-          <t>Merger/Acquisition: (NASD:RGEN) is acquiring BioLife Solutions in a deal expected to be completed soon, pending final closing conditions.</t>
+          <t>Merger/Acquisition: (NASD: SWKS) is acquiring Qorvo in a deal expected to be completed soon, pending final closing conditions.</t>
         </is>
       </c>
       <c r="J55" s="3" t="inlineStr">
         <is>
-          <t>https://www.prnewswire.com/news-releases/freshworks-set-to-join-sp-smallcap-600-302899001.html</t>
+          <t>https://www.prnewswire.com/news-releases/vylor-added-to-the-sp-500-twilio-set-to-join-sp-500-others-to-join-sp-midcap-400-and-sp-smallcap-600-302896675.html</t>
         </is>
       </c>
     </row>
@@ -3141,17 +3141,17 @@
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>Arcosa</t>
+          <t>BioLife Solutions</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>ACA</t>
+          <t>BLFS</t>
         </is>
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="E56" s="2" t="inlineStr"/>
@@ -3164,12 +3164,12 @@
       </c>
       <c r="I56" s="2" t="inlineStr">
         <is>
-          <t>Merger/Acquisition: S&amp;P 500 constituent CRH plc (NYSE: CRH ) has acquired Arcosa in a deal that closed today, October 23.</t>
+          <t>Merger/Acquisition: (NASD:RGEN) is acquiring BioLife Solutions in a deal expected to be completed soon, pending final closing conditions.</t>
         </is>
       </c>
       <c r="J56" s="3" t="inlineStr">
         <is>
-          <t>https://www.prnewswire.com/news-releases/howard-hughes-holdings-set-to-join-sp-smallcap-600-302918511.html</t>
+          <t>https://www.prnewswire.com/news-releases/freshworks-set-to-join-sp-smallcap-600-302899001.html</t>
         </is>
       </c>
     </row>
@@ -3181,17 +3181,17 @@
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>Supernus Pharmaceuticals</t>
+          <t>Arcosa</t>
         </is>
       </c>
       <c r="C57" s="2" t="inlineStr">
         <is>
-          <t>SUPN</t>
+          <t>ACA</t>
         </is>
       </c>
       <c r="D57" s="2" t="inlineStr">
         <is>
-          <t>2026-11-02</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="E57" s="2" t="inlineStr"/>
@@ -3204,12 +3204,12 @@
       </c>
       <c r="I57" s="2" t="inlineStr">
         <is>
-          <t>Merger/Acquisition: (NASD: INDV) is acquiring Supernus Pharmaceuticals in a deal expected to be completed soon, pending final closing conditions.</t>
+          <t>Merger/Acquisition: S&amp;P 500 constituent CRH plc (NYSE: CRH ) has acquired Arcosa in a deal that closed today, October 23.</t>
         </is>
       </c>
       <c r="J57" s="3" t="inlineStr">
         <is>
-          <t>https://www.prnewswire.com/news-releases/msg-rangers-and-huron-consulting-group-set-to-join-sp-smallcap-600-302917492.html</t>
+          <t>https://www.prnewswire.com/news-releases/howard-hughes-holdings-set-to-join-sp-smallcap-600-302918511.html</t>
         </is>
       </c>
     </row>
@@ -3231,7 +3231,7 @@
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>2026-11-03</t>
+          <t>2026-11-02</t>
         </is>
       </c>
       <c r="E58" s="2" t="inlineStr"/>
@@ -3244,12 +3244,92 @@
       </c>
       <c r="I58" s="2" t="inlineStr">
         <is>
+          <t>Merger/Acquisition: (NASD: INDV) is acquiring Supernus Pharmaceuticals in a deal expected to be completed soon, pending final closing conditions.</t>
+        </is>
+      </c>
+      <c r="J58" s="3" t="inlineStr">
+        <is>
+          <t>https://www.prnewswire.com/news-releases/msg-rangers-and-huron-consulting-group-set-to-join-sp-smallcap-600-302917492.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="inlineStr">
+        <is>
+          <t>S&amp;P 600</t>
+        </is>
+      </c>
+      <c r="B59" s="2" t="inlineStr">
+        <is>
+          <t>Supernus Pharmaceuticals</t>
+        </is>
+      </c>
+      <c r="C59" s="2" t="inlineStr">
+        <is>
+          <t>SUPN</t>
+        </is>
+      </c>
+      <c r="D59" s="2" t="inlineStr">
+        <is>
+          <t>2026-11-03</t>
+        </is>
+      </c>
+      <c r="E59" s="2" t="inlineStr"/>
+      <c r="F59" s="2" t="inlineStr"/>
+      <c r="G59" s="2" t="inlineStr"/>
+      <c r="H59" s="2" t="inlineStr">
+        <is>
+          <t>Removed, no matching addition found</t>
+        </is>
+      </c>
+      <c r="I59" s="2" t="inlineStr">
+        <is>
           <t>Merger/Acquisition: (NASD: INDV) is acquiring Supernus Pharmaceuticals in a transaction expected to close soon, subject to final closing conditions.</t>
         </is>
       </c>
-      <c r="J58" s="3" t="inlineStr">
+      <c r="J59" s="3" t="inlineStr">
         <is>
           <t>https://www.prnewswire.com/news-releases/updated-effective-date-huron-consulting-group-set-to-join-sp-smallcap-600-302922778.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="inlineStr">
+        <is>
+          <t>S&amp;P 600</t>
+        </is>
+      </c>
+      <c r="B60" s="2" t="inlineStr">
+        <is>
+          <t>LiveRamp Holdings</t>
+        </is>
+      </c>
+      <c r="C60" s="2" t="inlineStr">
+        <is>
+          <t>RAMP</t>
+        </is>
+      </c>
+      <c r="D60" s="2" t="inlineStr">
+        <is>
+          <t>2026-11-04</t>
+        </is>
+      </c>
+      <c r="E60" s="2" t="inlineStr"/>
+      <c r="F60" s="2" t="inlineStr"/>
+      <c r="G60" s="2" t="inlineStr"/>
+      <c r="H60" s="2" t="inlineStr">
+        <is>
+          <t>Removed, no matching addition found</t>
+        </is>
+      </c>
+      <c r="I60" s="2" t="inlineStr">
+        <is>
+          <t>Merger/Acquisition: Publicis Groupe SA (Euronext Paris: PUB) is acquiring LiveRamp Holdings in a deal expected to close soon, pending final closing conditions.</t>
+        </is>
+      </c>
+      <c r="J60" s="3" t="inlineStr">
+        <is>
+          <t>https://www.prnewswire.com/news-releases/okta-set-to-join-sp-500-others-to-join-sp-midcap-400-and-sp-smallcap-600-302925405.html</t>
         </is>
       </c>
     </row>
@@ -3312,6 +3392,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J56" r:id="rId55"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J57" r:id="rId56"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J58" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J59" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J60" r:id="rId59"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>